<commit_message>
[Nairne] 2025 GP reconciliation: remove TruQuant from expenses entirely
Per Nairne 2026-04-30: TruQuant is not a GP expense / 1099 recipient.
Even the August "Trader & Developer" $6,909.93 and "Spydr" $170.86
(Aug+Sep) — which the Distributions ledger tracked as TQ-bound payouts
inside the GP entity — are excluded. TQ's relationship is upstream of
Armada Prime Tech LLC.

Net effect: the ~$7,081 TQ-tagged amounts stay in GP retained earnings
and flow to K-1 net income.

Updated headline numbers:
- 2025 GP gross income (TPA-authoritative): $153,023.03 (unchanged)
- 2025 1099 payments: $139,541.45 (was $146,622.24)
- 2025 K-1 net income: -$79,637.36 (was -$86,718.15)
- Per-member K-1 (Raj/Nairne 50/50): -$38,871.71 each

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2025-armada-prime-tech-1099-k1.xlsx
+++ b/2025-armada-prime-tech-1099-k1.xlsx
@@ -554,7 +554,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>AUG ANOMALY: Aug used a different waterfall (9.5% Consultant + 13.5% Trader &amp; Developer + 5.5% Mgmt + 1.5% to principals = 30%). TruQuant moved upstream from Sep onwards. See 1099 Summary + Distributions Ledger tabs.</t>
+          <t>TruQuant payments excluded entirely (per Nairne 2026-04-30) — TQ is not a GP expense / 1099 recipient. Aug TQ-tagged ~$6,999 stays in retained earnings → flows to K-1 net income.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>60625.41</v>
+        <v>53544.62</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>146622.24</v>
+        <v>139541.45</v>
       </c>
       <c r="C14" s="7">
         <f> sum of all non-member contractor payments</f>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>-86718.15000000002</v>
+        <v>-79637.36000000002</v>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>-42412.10500000001</v>
+        <v>-38871.71000000001</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>-42412.10500000001</v>
+        <v>-38871.71000000001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -992,11 +992,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Trader &amp; Developer (TruQuant)</t>
+          <t>AJ Affleck</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>6909.93</v>
+        <v>4152.7</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1014,11 +1014,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AJ Affleck</t>
+          <t>Issac</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>4152.7</v>
+        <v>761.49</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1036,11 +1036,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Issac</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>761.49</v>
+        <v>164.9</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1056,75 +1056,31 @@
       <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Spydr (TruQuant)</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>170.86</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Individual 1099</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>From Distributions ledger (cash actually paid)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Luke</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>164.9</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Individual 1099</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>From Distributions ledger (cash actually paid)</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-    </row>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL 1099 PAYMENTS</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>139541.45</v>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+    </row>
+    <row r="13"/>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL 1099 PAYMENTS</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>146622.24</v>
-      </c>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Cross-check: 1099 total ($146,622.24) + Raj K-1 direct ($946.97) + Nairne K-1 direct ($946.97) = $148,516.18</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>Should approx equal Gross Perf Fees Crystallized (TPA): $153,023.03 — delta = $4,506.85 (= cash-vs-accrual timing + Aug TQ-T&amp;D treatment)</t>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Cross-check: 1099 total ($139,541.45) + Raj K-1 direct ($946.97) + Nairne K-1 direct ($946.97) = $141,435.39</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Should approx equal Gross Perf Fees Crystallized (TPA): $153,023.03 — delta = $11,587.64 (= cash-vs-accrual timing + Aug TQ-T&amp;D treatment)</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1205,10 +1161,10 @@
         <v>946.97</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>-43359.07500000001</v>
+        <v>-39818.68000000001</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>-42412.10500000001</v>
+        <v>-38871.71000000001</v>
       </c>
       <c r="E5" t="inlineStr"/>
     </row>
@@ -1222,10 +1178,10 @@
         <v>946.97</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>-43359.07500000001</v>
+        <v>-39818.68000000001</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>-42412.10500000001</v>
+        <v>-38871.71000000001</v>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
@@ -1247,7 +1203,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Less: 1099 contractor payments (incl. Fund Mgmt + Phil + consultants + Aug Trader &amp; Developer): $144,728.30</t>
+          <t>Less: 1099 contractor payments (incl. Fund Mgmt + Phil + consultants + Aug Trader &amp; Developer): $137,647.51</t>
         </is>
       </c>
     </row>
@@ -1267,14 +1223,14 @@
     </row>
     <row r="13">
       <c r="A13">
-        <f> GP Net Income (residual): $-86,718.15</f>
+        <f> GP Net Income (residual): $-79,637.36</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Per K-1 member (50/50): $-43,359.08</t>
+          <t>Per K-1 member (50/50): $-39,818.68</t>
         </is>
       </c>
     </row>
@@ -1307,10 +1263,18 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>TruQuant payments are excluded per Nairne 2026-04-30 (TQ is not a GP expense). Aug TQ-tagged ~$6,999 effectively flows into GP retained earnings → increases the K-1 net income line above.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A19:E19"/>
@@ -2420,11 +2384,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -2563,57 +2527,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Trader &amp; Developer (TruQuant)</t>
+          <t>AJ Affleck</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>6909.93</v>
+        <v>335.47</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0</v>
+        <v>285.77</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0</v>
+        <v>1268.23</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0</v>
+        <v>1833.52</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0</v>
+        <v>429.71</v>
       </c>
       <c r="G8" s="17" t="n">
-        <v>6909.93</v>
+        <v>4152.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AJ Affleck</t>
+          <t>Raj</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>335.47</v>
+        <v>255.92</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>285.77</v>
+        <v>62.32</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1268.23</v>
+        <v>262.24</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>1833.52</v>
+        <v>287.26</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>429.71</v>
+        <v>79.23</v>
       </c>
       <c r="G9" s="17" t="n">
-        <v>4152.7</v>
+        <v>946.97</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Raj</t>
+          <t>Nairne</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -2638,7 +2602,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nairne</t>
+          <t>Phil</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -2663,32 +2627,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Phil</t>
+          <t>Issac</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>255.92</v>
+        <v>0</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>62.32</v>
+        <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>262.24</v>
+        <v>254.12</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>287.26</v>
+        <v>785.85</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>79.23</v>
+        <v>-278.48</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>946.97</v>
+        <v>761.49</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Issac</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
@@ -2698,141 +2662,91 @@
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>254.12</v>
+        <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>785.85</v>
+        <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>-278.48</v>
+        <v>164.9</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>761.49</v>
+        <v>164.9</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Spydr (TruQuant)</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>88.78</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>82.08</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="17" t="n">
-        <v>170.86</v>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>MONTH TOTAL (cash actually paid out)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>8356.690000000001</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>12381.17</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>48583.18</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>56973.74000000001</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>15140.61</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>141435.39</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Luke</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>164.9</v>
-      </c>
-      <c r="G15" s="17" t="n">
-        <v>164.9</v>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TPA Perf Fees Crystallized (what was OWED)</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>15355.51</v>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>12474.75</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>51906.99</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>57074.08999999997</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>16211.69</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <v>153023.03</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>MONTH TOTAL (cash actually paid out)</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>15355.4</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>12463.25</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>48583.18</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>56973.74000000001</v>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>15140.61</v>
-      </c>
-      <c r="G16" s="12" t="n">
-        <v>148516.18</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>TPA Perf Fees Crystallized (what was OWED)</t>
-        </is>
-      </c>
-      <c r="B17" s="22" t="n">
-        <v>15355.51</v>
-      </c>
-      <c r="C17" s="22" t="n">
-        <v>12474.75</v>
-      </c>
-      <c r="D17" s="22" t="n">
-        <v>51906.99</v>
-      </c>
-      <c r="E17" s="22" t="n">
-        <v>57074.08999999997</v>
-      </c>
-      <c r="F17" s="22" t="n">
-        <v>16211.69</v>
-      </c>
-      <c r="G17" s="22" t="n">
-        <v>153023.03</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>DELTA (Owed - Paid; positive = unpaid liability)</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
-        <v>0.1100000000024011</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>11.50000000000182</v>
-      </c>
-      <c r="D18" s="13" t="n">
+      <c r="B16" s="13" t="n">
+        <v>6998.820000000002</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>93.58000000000175</v>
+      </c>
+      <c r="D16" s="13" t="n">
         <v>3323.809999999998</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E16" s="13" t="n">
         <v>100.3499999999622</v>
       </c>
-      <c r="F18" s="13" t="n">
+      <c r="F16" s="13" t="n">
         <v>1071.080000000004</v>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>4506.849999999977</v>
+      <c r="G16" s="13" t="n">
+        <v>11587.63999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Nairne] Add Nikki ($223 in Nov) to 1099 contractors
Per Nairne 2026-05-05: only Nikki approved from the 7-person delta list.
All others (Raj, Phil, Alec, Jake, Issac, Luke) remain at their original
Distributions ledger values. Doug Corpuz, Armada Prime Tech retained,
TruQuant, and Raj (Split) entries from the Updated file are NOT added.

Changes:
  - ACTUAL_PAID["2025-11"]["Nikki"] = 223.00
  - Added Nikki to P&L Direct Costs line and 1099 Recipients tab
  - Updated cover memo

Updated headline numbers:
  Revenue:          $153,023.03 (unchanged)
  1099 Contractors: $86,754.81  (was $86,531.81; +$223 Nikki)
  Op Expenses:      $91,225.00  (unchanged)
  Net Income GAAP:  $-24,956.78 (was $-24,733.78; -$223 Nikki)
  Net Income Reclass: $14,818.22 (was $15,041.22; -$223 Nikki)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2025-armada-prime-tech-1099-k1.xlsx
+++ b/2025-armada-prime-tech-1099-k1.xlsx
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>86531.81</v>
+        <v>86754.81</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>86531.81</v>
+        <v>86754.81</v>
       </c>
       <c r="C12" s="7" t="inlineStr"/>
     </row>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>-24733.78000000003</v>
+        <v>-24956.78000000003</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -859,15 +859,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Total cash out (1099s $86,531.81 + Nairne K-1 $34,188.88 + Raj K-1 $946.97 + Phil K-1 $946.97)</t>
+          <t>Total cash out (1099s $86,754.81 + Nairne K-1 $34,188.88 + Raj K-1 $946.97 + Phil K-1 $946.97)</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>122614.63</v>
+        <v>122837.63</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>vs Gross $153,023.03 — delta $30,408.40 (= retained / cash-vs-accrual / TQ exclusion)</t>
+          <t>vs Gross $153,023.03 — delta $30,185.40 (= retained / cash-vs-accrual / TQ exclusion)</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2661,173 +2661,192 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Nikki</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1099</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>1099 Subtotal</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="8" t="n">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="8" t="n">
         <v>21928.06</v>
       </c>
-      <c r="D22" s="8" t="n">
-        <v>36661.7</v>
-      </c>
-      <c r="E22" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="D23" s="8" t="n">
+        <v>36884.7</v>
+      </c>
+      <c r="E23" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>TOTAL CASH PAID TO PEOPLE (K-1 + 1099)</t>
         </is>
       </c>
-      <c r="D24" s="17" t="n">
-        <v>52767.23</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="33" t="inlineStr">
+      <c r="D25" s="17" t="n">
+        <v>52990.23</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>OPERATING EXPENSES (paid by GP entity to vendors)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Chris</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Payroll/Contractor</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>7500</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alpha Verification</t>
+          <t>Chris</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Verification/Compliance</t>
+          <t>Payroll/Contractor</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>2250</v>
+        <v>7500</v>
       </c>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Alpha Verification</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Verification/Compliance</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Formidium (TPA)</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Admin / TPA Fee</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C31" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>VERIFY GP-paid vs fund-paid</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Op Expenses Subtotal</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="8" t="n">
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="8" t="n">
         <v>10350</v>
       </c>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="33" t="inlineStr">
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
         <is>
           <t>RECONCILIATION</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Capital In (TPA Perf Fees Crystallized)</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="n">
-        <v>57074.08999999997</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Less: Cash to people (K-1 + 1099)</t>
+          <t>Capital In (TPA Perf Fees Crystallized)</t>
         </is>
       </c>
       <c r="D35" s="6" t="n">
-        <v>-52767.23</v>
+        <v>57074.08999999997</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Less: Cash to people (K-1 + 1099)</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>-52990.23</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Less: Op expenses to vendors</t>
         </is>
       </c>
-      <c r="D36" s="6" t="n">
+      <c r="D37" s="6" t="n">
         <v>-10350</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="7">
+    <row r="38">
+      <c r="A38" s="7">
         <f> Residual / (Deficit) for the month</f>
         <v/>
       </c>
-      <c r="B37" s="34" t="n"/>
-      <c r="C37" s="34" t="n"/>
-      <c r="D37" s="35" t="n">
-        <v>-6043.140000000029</v>
-      </c>
-      <c r="E37" s="34" t="n"/>
+      <c r="B38" s="34" t="n"/>
+      <c r="C38" s="34" t="n"/>
+      <c r="D38" s="35" t="n">
+        <v>-6266.140000000029</v>
+      </c>
+      <c r="E38" s="34" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3509,7 +3528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3658,11 +3677,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Nikki</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>164.9</v>
+        <v>223</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -3678,31 +3697,53 @@
       <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Individual 1099</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>From Distributions ledger (cash actually paid)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>TOTAL 1099 PAYMENTS</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
-        <v>86531.81</v>
-      </c>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>K-1 partner cash distributions (NOT on 1099s): Nairne $34,188.88 + Raj $946.97 = $35,135.85</t>
-        </is>
-      </c>
-    </row>
+      <c r="B11" s="12" t="n">
+        <v>86754.81</v>
+      </c>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Cross-check: 1099 total ($86,531.81) + K-1 cash ($35,135.85) = $121,667.66; Gross perf fees per TPA = $153,023.03; delta = $31,355.37 (cash-vs-accrual timing + Aug TQ-T&amp;D excluded)</t>
+          <t>K-1 partner cash distributions (NOT on 1099s): Nairne $34,188.88 + Raj $946.97 = $35,135.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Cross-check: 1099 total ($86,754.81) + K-1 cash ($35,135.85) = $121,890.66; Gross perf fees per TPA = $153,023.03; delta = $31,132.37 (cash-vs-accrual timing + Aug TQ-T&amp;D excluded)</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3829,7 @@
         <v>34188.88</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>-24328.30819672134</v>
+        <v>-24547.65245901642</v>
       </c>
       <c r="E5" t="inlineStr"/>
     </row>
@@ -3807,7 +3848,7 @@
         <v>946.97</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>-202.7359016393445</v>
+        <v>-204.5637704918035</v>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
@@ -3826,7 +3867,7 @@
         <v>946.97</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>-202.7359016393445</v>
+        <v>-204.5637704918035</v>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
@@ -3848,7 +3889,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Less: 1099 contractor expenses (Alec/Jake/AJ/Issac/Luke): $86,531.81</t>
+          <t>Less: 1099 contractor expenses (Alec/Jake/AJ/Issac/Luke): $86,754.81</t>
         </is>
       </c>
     </row>
@@ -3861,28 +3902,28 @@
     </row>
     <row r="13">
       <c r="A13">
-        <f> Partnership NET INCOME (allocated to K-1s): $-24,733.78</f>
+        <f> Partnership NET INCOME (allocated to K-1s): $-24,956.78</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nairne allocated share (98.36%): $-24,328.31</t>
+          <t>Nairne allocated share (98.36%): $-24,547.65</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Raj allocated share (0.82%): $-202.74</t>
+          <t>Raj allocated share (0.82%): $-204.56</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Phil allocated share (0.82%): $-202.74</t>
+          <t>Phil allocated share (0.82%): $-204.56</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5296,7 +5337,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Nikki</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
@@ -5309,113 +5350,138 @@
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
+        <v>223</v>
+      </c>
+      <c r="F12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="G12" s="17" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="6" t="n">
         <v>164.9</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G13" s="17" t="n">
         <v>164.9</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Fund Mgmt 59.5% (= Nairne K-1)</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="24" t="n">
+      <c r="G14" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>MONTH TOTAL (cash actually paid out)</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B15" s="12" t="n">
         <v>8356.68</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C15" s="12" t="n">
         <v>16531.16</v>
       </c>
-      <c r="D14" s="12" t="n">
+      <c r="D15" s="12" t="n">
         <v>29591.02</v>
       </c>
-      <c r="E14" s="12" t="n">
-        <v>52767.23</v>
-      </c>
-      <c r="F14" s="12" t="n">
+      <c r="E15" s="12" t="n">
+        <v>52990.23</v>
+      </c>
+      <c r="F15" s="12" t="n">
         <v>15368.54</v>
       </c>
-      <c r="G14" s="12" t="n">
-        <v>122614.63</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="G15" s="12" t="n">
+        <v>122837.63</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>TPA Perf Fees Crystallized (what was OWED)</t>
         </is>
       </c>
-      <c r="B15" s="25" t="n">
+      <c r="B16" s="25" t="n">
         <v>15355.51</v>
       </c>
-      <c r="C15" s="25" t="n">
+      <c r="C16" s="25" t="n">
         <v>12474.75</v>
       </c>
-      <c r="D15" s="25" t="n">
+      <c r="D16" s="25" t="n">
         <v>51906.99</v>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E16" s="25" t="n">
         <v>57074.08999999997</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F16" s="25" t="n">
         <v>16211.69</v>
       </c>
-      <c r="G15" s="25" t="n">
+      <c r="G16" s="25" t="n">
         <v>153023.03</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>DELTA (Owed - Paid; positive = unpaid liability)</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B17" s="13" t="n">
         <v>6998.830000000002</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C17" s="13" t="n">
         <v>-4056.409999999998</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D17" s="13" t="n">
         <v>22315.97</v>
       </c>
-      <c r="E16" s="13" t="n">
-        <v>4306.859999999964</v>
-      </c>
-      <c r="F16" s="13" t="n">
+      <c r="E17" s="13" t="n">
+        <v>4083.859999999964</v>
+      </c>
+      <c r="F17" s="13" t="n">
         <v>843.1500000000015</v>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>30408.39999999997</v>
+      <c r="G17" s="13" t="n">
+        <v>30185.39999999997</v>
       </c>
     </row>
   </sheetData>
@@ -5835,7 +5901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -6282,7 +6348,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Nikki</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6299,248 +6365,281 @@
       <c r="H13" s="30" t="n">
         <v>0</v>
       </c>
+      <c r="I13" s="6" t="n">
+        <v>223</v>
+      </c>
       <c r="J13" s="30" t="n">
+        <v>223</v>
+      </c>
+      <c r="L13" s="30" t="n">
+        <v>223</v>
+      </c>
+      <c r="M13" s="17" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1099</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="F14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="6" t="n">
         <v>164.9</v>
       </c>
-      <c r="L13" s="30" t="n">
+      <c r="L14" s="30" t="n">
         <v>164.9</v>
       </c>
-      <c r="M13" s="17" t="n">
+      <c r="M14" s="17" t="n">
         <v>164.9</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>K-1 SUBTOTAL (Nairne + Raj + Phil)</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>K-1</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>2175.34</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>2175.34</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>5969.759999999999</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>8145.099999999999</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>6769.129999999999</v>
-      </c>
-      <c r="H14" s="12" t="n">
-        <v>14914.23</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>16105.53</v>
-      </c>
-      <c r="J14" s="12" t="n">
-        <v>31019.76</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>5063.059999999999</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>36082.82</v>
-      </c>
-      <c r="M14" s="12" t="n">
-        <v>36082.82</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
+          <t>K-1 SUBTOTAL (Nairne + Raj + Phil)</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>K-1</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>2175.34</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>2175.34</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>5969.759999999999</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>8145.099999999999</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>6769.129999999999</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>14914.23</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>16105.53</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>31019.76</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>5063.059999999999</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>36082.82</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>36082.82</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
           <t>1099 SUBTOTAL (consultants only)</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>1099</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C16" s="12" t="n">
         <v>6181.34</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D16" s="12" t="n">
         <v>6181.34</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E16" s="12" t="n">
         <v>10561.4</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F16" s="12" t="n">
         <v>16742.74</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="G16" s="12" t="n">
         <v>22821.89</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H16" s="12" t="n">
         <v>39564.63</v>
       </c>
-      <c r="I15" s="12" t="n">
-        <v>36661.7</v>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>76226.32999999999</v>
-      </c>
-      <c r="K15" s="12" t="n">
+      <c r="I16" s="12" t="n">
+        <v>36884.7</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>76449.32999999999</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>10305.48</v>
       </c>
-      <c r="L15" s="12" t="n">
-        <v>86531.80999999998</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>86531.80999999998</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="L16" s="12" t="n">
+        <v>86754.80999999998</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>86754.80999999998</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>GRAND TOTAL (K-1 + 1099)</t>
         </is>
       </c>
-      <c r="B16" s="31" t="inlineStr"/>
-      <c r="C16" s="32" t="n">
+      <c r="B17" s="31" t="inlineStr"/>
+      <c r="C17" s="32" t="n">
         <v>8356.68</v>
       </c>
-      <c r="D16" s="32" t="n">
+      <c r="D17" s="32" t="n">
         <v>8356.68</v>
       </c>
-      <c r="E16" s="32" t="n">
+      <c r="E17" s="32" t="n">
         <v>16531.16</v>
       </c>
-      <c r="F16" s="32" t="n">
+      <c r="F17" s="32" t="n">
         <v>24887.84</v>
       </c>
-      <c r="G16" s="32" t="n">
+      <c r="G17" s="32" t="n">
         <v>29591.02</v>
       </c>
-      <c r="H16" s="32" t="n">
+      <c r="H17" s="32" t="n">
         <v>54478.86</v>
       </c>
-      <c r="I16" s="32" t="n">
-        <v>52767.23</v>
-      </c>
-      <c r="J16" s="32" t="n">
-        <v>107246.09</v>
-      </c>
-      <c r="K16" s="32" t="n">
+      <c r="I17" s="32" t="n">
+        <v>52990.23</v>
+      </c>
+      <c r="J17" s="32" t="n">
+        <v>107469.09</v>
+      </c>
+      <c r="K17" s="32" t="n">
         <v>15368.54</v>
       </c>
-      <c r="L16" s="32" t="n">
-        <v>122614.63</v>
-      </c>
-      <c r="M16" s="32" t="n">
-        <v>122614.63</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>TPA Perf Fees Crystallized (Gross GP Income)</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="25" t="n">
-        <v>15355.51</v>
-      </c>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="25" t="n">
-        <v>12474.75</v>
-      </c>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="25" t="n">
-        <v>51906.99</v>
-      </c>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="25" t="n">
-        <v>57074.08999999997</v>
-      </c>
-      <c r="J17" s="10" t="n"/>
-      <c r="K17" s="25" t="n">
-        <v>16211.69</v>
-      </c>
-      <c r="L17" s="10" t="n"/>
-      <c r="M17" s="25" t="n">
-        <v>153023.03</v>
+      <c r="L17" s="32" t="n">
+        <v>122837.63</v>
+      </c>
+      <c r="M17" s="32" t="n">
+        <v>122837.63</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Op Expenses (paid from GP retained)</t>
+          <t>TPA Perf Fees Crystallized (Gross GP Income)</t>
         </is>
       </c>
       <c r="B18" s="10" t="n"/>
       <c r="C18" s="25" t="n">
-        <v>10275</v>
+        <v>15355.51</v>
       </c>
       <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
+      <c r="E18" s="25" t="n">
+        <v>12474.75</v>
+      </c>
       <c r="F18" s="10" t="n"/>
       <c r="G18" s="25" t="n">
-        <v>43500</v>
+        <v>51906.99</v>
       </c>
       <c r="H18" s="10" t="n"/>
       <c r="I18" s="25" t="n">
-        <v>10350</v>
+        <v>57074.08999999997</v>
       </c>
       <c r="J18" s="10" t="n"/>
       <c r="K18" s="25" t="n">
-        <v>27100</v>
+        <v>16211.69</v>
       </c>
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="25" t="n">
+        <v>153023.03</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Op Expenses (paid from GP retained)</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="25" t="n">
+        <v>10275</v>
+      </c>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="25" t="n">
+        <v>43500</v>
+      </c>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="25" t="n">
+        <v>10350</v>
+      </c>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="25" t="n">
+        <v>27100</v>
+      </c>
+      <c r="L19" s="10" t="n"/>
+      <c r="M19" s="25" t="n">
         <v>91225</v>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>NOTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="35" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Payouts shown are NET — already after weighted costs (per Nairne 2026-04-30). The Distributions ledger's separate 'Gross vs Net' table tracks cumulative settlement balances (carries forward unpaid amounts) and a layer of Coinbase/wire/Crypto fees (~2.8%) plus per-person 'Expense' allocations (Nairne Expense, Alec Expense, etc.) — those are nested inside the Net amounts you see here.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="35" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>TruQuant payments are excluded entirely (per Nairne 2026-04-30). The Aug TruQuant amounts ($6,909.93 Trader &amp; Developer + $88.78 Spydr) and Sep Spydr $82.08 are NOT in any of the rows above.</t>
+          <t>Payouts shown are NET — already after weighted costs (per Nairne 2026-04-30). The Distributions ledger's separate 'Gross vs Net' table tracks cumulative settlement balances (carries forward unpaid amounts) and a layer of Coinbase/wire/Crypto fees (~2.8%) plus per-person 'Expense' allocations (Nairne Expense, Alec Expense, etc.) — those are nested inside the Net amounts you see here.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="35" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>Aug 2025 used a different waterfall (Fund Mgmt was 5.5% not 59.5%). From Sep onwards: standard 59.5% Mgmt + 39% Consultant + 0.5%×3 principals.</t>
+          <t>TruQuant payments are excluded entirely (per Nairne 2026-04-30). The Aug TruQuant amounts ($6,909.93 Trader &amp; Developer + $88.78 Spydr) and Sep Spydr $82.08 are NOT in any of the rows above.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="35" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Issac shows -$278.48 in Dec — clawback against prior month overpayment.</t>
+          <t>Aug 2025 used a different waterfall (Fund Mgmt was 5.5% not 59.5%). From Sep onwards: standard 59.5% Mgmt + 39% Consultant + 0.5%×3 principals.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="35" customHeight="1">
       <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Issac shows -$278.48 in Dec — clawback against prior month overpayment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Op Expenses row at the bottom is the GP-paid vendor expenses (not allocated to individuals on this tab — see Monthly Op Expenses tab for vendor breakdown).</t>
         </is>
@@ -6551,7 +6650,7 @@
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A23:M23"/>
     <mergeCell ref="A22:M22"/>
-    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="A26:M26"/>
     <mergeCell ref="A25:M25"/>
     <mergeCell ref="A24:M24"/>
     <mergeCell ref="A2:M2"/>

</xml_diff>